<commit_message>
Point PDF and header steps to the job instruction sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFKV7Fk6B8YhD5sjA3vqAV
</commit_message>
<xml_diff>
--- a/GAR_Booklet_process_playbook.xlsx
+++ b/GAR_Booklet_process_playbook.xlsx
@@ -828,7 +828,7 @@
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>1) Perform the same checks as in step 1.4, now in Tangelo.
-2) Check that the front cover and all headers show the current quarter.</t>
+2) Update and check the headers as described in the job instruction sheet (step 5 of “Steps to upload and synchronize the excel file”).</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Follow the job instruction sheet, section “Steps to generate the pdf” (formatting check, nothing hidden or cut, headers on current quarter). Save the PDF in the quarter folder using the naming convention of previous quarters.</t>
+          <t>Follow the job instruction sheet, section “Steps to generate the pdf”. Save the PDF in the quarter folder using the naming convention of previous quarters.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add short Tangelo summaries with reference to the job instruction sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFKV7Fk6B8YhD5sjA3vqAV
</commit_message>
<xml_diff>
--- a/GAR_Booklet_process_playbook.xlsx
+++ b/GAR_Booklet_process_playbook.xlsx
@@ -620,7 +620,8 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Follow the job instruction sheet, section “How to create the presentation for the new quarter”.</t>
+          <t>In Tangelo, copy last quarter's booklet, keep the GAR booklet data source, rename the copy to the new quarter (description field) and save.
+For details and screenshots, see the job instruction sheet, section “How to create the presentation for the new quarter”.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -774,7 +775,8 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Follow the job instruction sheet, section “Steps to upload and synchronize the excel file”.</t>
+          <t>In Tangelo, go to Data source → GAR Booklet, select the new Excel file and click play until the bar is green and shows “ready”. Then open the booklet and click both synchronise buttons until the line turns green.
+For details and screenshots, see the job instruction sheet, section “Steps to upload and synchronize the excel file” (steps 1–4).</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -828,7 +830,8 @@
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>1) Perform the same checks as in step 1.4, now in Tangelo.
-2) Update and check the headers as described in the job instruction sheet (step 5 of “Steps to upload and synchronize the excel file”).</t>
+2) Update the front cover header to the current quarter and check all headers.
+For details, see the job instruction sheet, section “Steps to upload and synchronize the excel file” (step 5).</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1058,7 +1061,8 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Follow the job instruction sheet, section “Steps to generate the pdf”. Save the PDF in the quarter folder using the naming convention of previous quarters.</t>
+          <t>Check the formatting (no tables split over two pages, nothing hidden or cut, headers on the current quarter), then generate the PDF in Tangelo with the Acrobat button. Save the PDF in the quarter folder using the naming convention of previous quarters.
+For details, see the job instruction sheet, section “Steps to generate the pdf”.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">

</xml_diff>